<commit_message>
Reupload missing adds in git, working well
</commit_message>
<xml_diff>
--- a/src/main/resources/Simple_Chocolate_Cake_Ingredients.xlsx
+++ b/src/main/resources/Simple_Chocolate_Cake_Ingredients.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="i cannot access the xlsx file y" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Ingredient" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t xml:space="preserve">Ingredient</t>
   </si>
@@ -28,13 +28,10 @@
     <t xml:space="preserve">Quantity</t>
   </si>
   <si>
-    <t xml:space="preserve">Price (EUR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price (MGA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAX &amp; impôts</t>
+    <t xml:space="preserve">Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAX</t>
   </si>
   <si>
     <t xml:space="preserve">All-purpose flour</t>
@@ -43,76 +40,73 @@
     <t xml:space="preserve">1 1/2 cups (190g)</t>
   </si>
   <si>
-    <t xml:space="preserve">2,000 MGA</t>
-  </si>
-  <si>
     <t xml:space="preserve">Granulated sugar</t>
   </si>
   <si>
     <t xml:space="preserve">1 cup (200g)</t>
   </si>
   <si>
-    <t xml:space="preserve">1,750 MGA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unsweetened cocoa powder</t>
+    <t xml:space="preserve">Cocoa powder</t>
   </si>
   <si>
     <t xml:space="preserve">3/4 cup (75g)</t>
   </si>
   <si>
-    <t xml:space="preserve">3,250 MGA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baking soda</t>
+    <t xml:space="preserve">Baking Soda</t>
   </si>
   <si>
     <t xml:space="preserve">1 teaspoon</t>
   </si>
   <si>
-    <t xml:space="preserve">250 MGA</t>
-  </si>
-  <si>
     <t xml:space="preserve">Baking powder</t>
   </si>
   <si>
+    <t xml:space="preserve">Eggs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 large</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vegetable oil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/2 cup (120ml)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Milk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 cup (240ml)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vanilla extract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chocolat Powder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 teaspoon</t>
+  </si>
+  <si>
     <t xml:space="preserve">Salt</t>
   </si>
   <si>
     <t xml:space="preserve">1/2 teaspoon</t>
   </si>
   <si>
-    <t xml:space="preserve">100 MGA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eggs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 large</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,000 MGA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vegetable oil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1/2 cup (120ml)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,250 MGA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Milk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 cup (240ml)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,000 MGA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vanilla extract</t>
+    <t xml:space="preserve">Unsalted Butter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/4 cup (275g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lemon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carrot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strawberry</t>
   </si>
 </sst>
 </file>
@@ -197,24 +191,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -407,201 +405,265 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="0"/>
+    </row>
+    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0.1499</v>
+      </c>
+      <c r="E2" s="0"/>
+    </row>
+    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>0.1499</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="C3" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.2399</v>
+      </c>
+      <c r="E3" s="0"/>
+    </row>
+    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="C4" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E4" s="0"/>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="n">
-        <v>0.2399</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C5" s="4" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.2999</v>
+      </c>
+      <c r="E5" s="0"/>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0.2999</v>
+      </c>
+      <c r="E6" s="0"/>
+    </row>
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C7" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="0"/>
+    </row>
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>0.2999</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="C8" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>0.2999</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C9" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.1299</v>
+      </c>
+      <c r="E9" s="0"/>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>0.0349</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>0.28</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>0.1299</v>
-      </c>
+      <c r="B10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0.1799</v>
+      </c>
+      <c r="E10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="5" t="n">
         <v>0.1799</v>
       </c>
+      <c r="E11" s="0"/>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0.0349</v>
+      </c>
+      <c r="E12" s="0"/>
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.0349</v>
+      </c>
+      <c r="E13" s="0"/>
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0.0799</v>
+      </c>
+      <c r="E14" s="0"/>
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0.0899</v>
+      </c>
+      <c r="E15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0.0499</v>
+      </c>
+      <c r="E16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0"/>
+      <c r="B17" s="0"/>
+      <c r="C17" s="0"/>
+      <c r="D17" s="0"/>
+      <c r="E17" s="0"/>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0"/>
+      <c r="B18" s="0"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C19" s="4"/>
+      <c r="E19" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>